<commit_message>
Bring down coal RAF to previous value
</commit_message>
<xml_diff>
--- a/InputData/elec/RAF/Regional Availability Factor.xlsx
+++ b/InputData/elec/RAF/Regional Availability Factor.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us\InputData\elec\RAF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F62B5974-9E73-457B-905F-7DA1D40EE2A1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{84A8C125-1BDA-4536-BA95-3365DBDBC4D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
   </bookViews>
@@ -1186,82 +1186,82 @@
         <v>0.8</v>
       </c>
       <c r="C2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="D2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="F2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="J2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="K2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="M2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="N2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="O2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="P2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="R2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="S2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="T2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="U2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="V2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="W2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="X2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Y2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Z2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="AA2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="AB2">
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="3" spans="1:28" x14ac:dyDescent="0.35">
@@ -2220,107 +2220,107 @@
       </c>
       <c r="C14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="D14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="E14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="F14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="G14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="H14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="I14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="J14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="K14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="L14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="M14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="N14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="O14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="P14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Q14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="R14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="S14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="T14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="U14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="V14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="W14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="X14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Y14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="Z14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="AA14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
       <c r="AB14">
         <f t="shared" si="0"/>
-        <v>0.8</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="15" spans="1:28" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
RAF updates via calibration
</commit_message>
<xml_diff>
--- a/InputData/elec/RAF/Regional Availability Factor.xlsx
+++ b/InputData/elec/RAF/Regional Availability Factor.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RobbieOrvis\Models\US\Models\eps-us\InputData\elec\RAF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9841894-88E4-4415-8A7E-DD2FE4CFDB7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFF73A49-FEDC-4BBB-BCB2-03B2ADBAAE48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" activeTab="1" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="57840" windowHeight="23520" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -601,9 +601,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
-    <a:clrScheme name="Office 2013 - 2022">
+    <a:clrScheme name="Office">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -641,7 +641,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office 2013 - 2022">
+    <a:fontScheme name="Office">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -747,7 +747,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office 2013 - 2022">
+    <a:fmtScheme name="Office">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -889,7 +889,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1092,185 +1092,179 @@
   <sheetPr>
     <tabColor theme="4" tint="-0.499984740745262"/>
   </sheetPr>
-  <dimension ref="A1:AB25"/>
+  <dimension ref="A1:AA25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="34.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:28">
+    <row r="1" spans="1:27">
       <c r="A1" t="s">
         <v>22</v>
       </c>
       <c r="B1" s="3">
-        <v>2024</v>
+        <v>2025</v>
       </c>
       <c r="C1">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="D1">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="E1">
-        <v>2027</v>
+        <v>2028</v>
       </c>
       <c r="F1">
-        <v>2028</v>
+        <v>2029</v>
       </c>
       <c r="G1">
-        <v>2029</v>
+        <v>2030</v>
       </c>
       <c r="H1">
-        <v>2030</v>
+        <v>2031</v>
       </c>
       <c r="I1">
-        <v>2031</v>
+        <v>2032</v>
       </c>
       <c r="J1">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="K1">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="L1">
-        <v>2034</v>
+        <v>2035</v>
       </c>
       <c r="M1">
-        <v>2035</v>
+        <v>2036</v>
       </c>
       <c r="N1">
-        <v>2036</v>
+        <v>2037</v>
       </c>
       <c r="O1">
-        <v>2037</v>
+        <v>2038</v>
       </c>
       <c r="P1">
-        <v>2038</v>
+        <v>2039</v>
       </c>
       <c r="Q1">
-        <v>2039</v>
+        <v>2040</v>
       </c>
       <c r="R1">
-        <v>2040</v>
+        <v>2041</v>
       </c>
       <c r="S1">
-        <v>2041</v>
+        <v>2042</v>
       </c>
       <c r="T1">
-        <v>2042</v>
+        <v>2043</v>
       </c>
       <c r="U1">
-        <v>2043</v>
+        <v>2044</v>
       </c>
       <c r="V1">
-        <v>2044</v>
+        <v>2045</v>
       </c>
       <c r="W1">
-        <v>2045</v>
+        <v>2046</v>
       </c>
       <c r="X1">
-        <v>2046</v>
+        <v>2047</v>
       </c>
       <c r="Y1">
-        <v>2047</v>
+        <v>2048</v>
       </c>
       <c r="Z1">
-        <v>2048</v>
+        <v>2049</v>
       </c>
       <c r="AA1">
-        <v>2049</v>
-      </c>
-      <c r="AB1">
         <v>2050</v>
       </c>
     </row>
-    <row r="2" spans="1:28">
+    <row r="2" spans="1:27">
       <c r="A2" t="s">
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.9</v>
+        <v>0.63</v>
       </c>
       <c r="C2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="D2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="E2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="F2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="G2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="H2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="I2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="J2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="K2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="L2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="M2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="N2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="O2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="P2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="Q2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="R2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="S2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="T2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="U2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="V2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="W2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="X2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="Y2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="Z2">
-        <v>0.6</v>
+        <v>0.63</v>
       </c>
       <c r="AA2">
-        <v>0.6</v>
-      </c>
-      <c r="AB2">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:28">
+        <v>0.63</v>
+      </c>
+    </row>
+    <row r="3" spans="1:27">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -1352,11 +1346,8 @@
       <c r="AA3">
         <v>0.9</v>
       </c>
-      <c r="AB3">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="4" spans="1:28">
+    </row>
+    <row r="4" spans="1:27">
       <c r="A4" t="s">
         <v>62</v>
       </c>
@@ -1438,11 +1429,8 @@
       <c r="AA4">
         <v>0.9</v>
       </c>
-      <c r="AB4">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="5" spans="1:28">
+    </row>
+    <row r="5" spans="1:27">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -1524,11 +1512,8 @@
       <c r="AA5">
         <v>1</v>
       </c>
-      <c r="AB5">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:28">
+    </row>
+    <row r="6" spans="1:27">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -1610,11 +1595,8 @@
       <c r="AA6">
         <v>1</v>
       </c>
-      <c r="AB6">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7" spans="1:28">
+    </row>
+    <row r="7" spans="1:27">
       <c r="A7" t="s">
         <v>5</v>
       </c>
@@ -1696,11 +1678,8 @@
       <c r="AA7">
         <v>1</v>
       </c>
-      <c r="AB7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8" spans="1:28">
+    </row>
+    <row r="8" spans="1:27">
       <c r="A8" t="s">
         <v>6</v>
       </c>
@@ -1782,11 +1761,8 @@
       <c r="AA8">
         <v>1</v>
       </c>
-      <c r="AB8">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9" spans="1:28">
+    </row>
+    <row r="9" spans="1:27">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -1868,11 +1844,8 @@
       <c r="AA9">
         <v>1</v>
       </c>
-      <c r="AB9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:28">
+    </row>
+    <row r="10" spans="1:27">
       <c r="A10" t="s">
         <v>8</v>
       </c>
@@ -1954,11 +1927,8 @@
       <c r="AA10">
         <v>1</v>
       </c>
-      <c r="AB10">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:28">
+    </row>
+    <row r="11" spans="1:27">
       <c r="A11" t="s">
         <v>9</v>
       </c>
@@ -2040,11 +2010,8 @@
       <c r="AA11">
         <v>1</v>
       </c>
-      <c r="AB11">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:28">
+    </row>
+    <row r="12" spans="1:27">
       <c r="A12" t="s">
         <v>10</v>
       </c>
@@ -2126,11 +2093,8 @@
       <c r="AA12">
         <v>0.9</v>
       </c>
-      <c r="AB12">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="13" spans="1:28">
+    </row>
+    <row r="13" spans="1:27">
       <c r="A13" t="s">
         <v>11</v>
       </c>
@@ -2212,124 +2176,91 @@
       <c r="AA13">
         <v>0.9</v>
       </c>
-      <c r="AB13">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:28">
+    </row>
+    <row r="14" spans="1:27">
       <c r="A14" t="s">
         <v>12</v>
       </c>
       <c r="B14">
-        <f>B2</f>
-        <v>0.9</v>
+        <v>0.6</v>
       </c>
       <c r="C14">
-        <f t="shared" ref="C14:AB14" si="0">C2</f>
         <v>0.6</v>
       </c>
       <c r="D14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="E14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="F14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="G14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="H14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="I14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="J14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="K14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="L14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="M14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="N14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="O14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="P14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="Q14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="R14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="S14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="T14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="U14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="V14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="W14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="X14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="Y14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="Z14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
       <c r="AA14">
-        <f t="shared" si="0"/>
         <v>0.6</v>
       </c>
-      <c r="AB14">
-        <f t="shared" si="0"/>
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="15" spans="1:28">
+    </row>
+    <row r="15" spans="1:27">
       <c r="A15" t="s">
         <v>13</v>
       </c>
@@ -2411,11 +2342,8 @@
       <c r="AA15">
         <v>1</v>
       </c>
-      <c r="AB15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:28">
+    </row>
+    <row r="16" spans="1:27">
       <c r="A16" t="s">
         <v>14</v>
       </c>
@@ -2497,11 +2425,8 @@
       <c r="AA16">
         <v>1</v>
       </c>
-      <c r="AB16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:28">
+    </row>
+    <row r="17" spans="1:27">
       <c r="A17" t="s">
         <v>15</v>
       </c>
@@ -2583,11 +2508,8 @@
       <c r="AA17">
         <v>1</v>
       </c>
-      <c r="AB17">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:28">
+    </row>
+    <row r="18" spans="1:27">
       <c r="A18" t="s">
         <v>16</v>
       </c>
@@ -2669,11 +2591,8 @@
       <c r="AA18">
         <v>1</v>
       </c>
-      <c r="AB18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:28">
+    </row>
+    <row r="19" spans="1:27">
       <c r="A19" t="s">
         <v>17</v>
       </c>
@@ -2755,11 +2674,8 @@
       <c r="AA19">
         <v>0.9</v>
       </c>
-      <c r="AB19">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="20" spans="1:28">
+    </row>
+    <row r="20" spans="1:27">
       <c r="A20" t="s">
         <v>18</v>
       </c>
@@ -2841,11 +2757,8 @@
       <c r="AA20">
         <v>0.9</v>
       </c>
-      <c r="AB20">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="21" spans="1:28">
+    </row>
+    <row r="21" spans="1:27">
       <c r="A21" t="s">
         <v>19</v>
       </c>
@@ -2927,11 +2840,8 @@
       <c r="AA21">
         <v>0.9</v>
       </c>
-      <c r="AB21">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="22" spans="1:28">
+    </row>
+    <row r="22" spans="1:27">
       <c r="A22" t="s">
         <v>20</v>
       </c>
@@ -3013,11 +2923,8 @@
       <c r="AA22">
         <v>0.9</v>
       </c>
-      <c r="AB22">
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="23" spans="1:28">
+    </row>
+    <row r="23" spans="1:27">
       <c r="A23" t="s">
         <v>21</v>
       </c>
@@ -3099,233 +3006,170 @@
       <c r="AA23">
         <v>1</v>
       </c>
-      <c r="AB23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:28">
+    </row>
+    <row r="24" spans="1:27">
       <c r="A24" t="s">
         <v>45</v>
       </c>
       <c r="B24">
-        <f>B13</f>
         <v>0.9</v>
       </c>
       <c r="C24">
-        <f t="shared" ref="C24:AB24" si="1">C13</f>
         <v>0.9</v>
       </c>
       <c r="D24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="E24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="F24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="G24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="H24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="I24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="J24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="K24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="L24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="M24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="N24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="O24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="P24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="Q24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="R24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="S24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="T24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="U24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="V24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="W24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="X24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="Y24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="Z24">
-        <f t="shared" si="1"/>
         <v>0.9</v>
       </c>
       <c r="AA24">
-        <f t="shared" si="1"/>
-        <v>0.9</v>
-      </c>
-      <c r="AB24">
-        <f t="shared" si="1"/>
-        <v>0.9</v>
-      </c>
-    </row>
-    <row r="25" spans="1:28">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="25" spans="1:27">
       <c r="A25" t="s">
         <v>46</v>
       </c>
       <c r="B25">
-        <f>B4</f>
         <v>0.9</v>
       </c>
       <c r="C25">
-        <f t="shared" ref="C25:AB25" si="2">C4</f>
         <v>0.9</v>
       </c>
       <c r="D25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="E25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="F25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="G25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="H25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="I25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="J25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="K25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="L25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="M25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="N25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="O25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="P25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="Q25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="R25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="S25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="T25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="U25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="V25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="W25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="X25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="Y25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="Z25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
       <c r="AA25">
-        <f t="shared" si="2"/>
-        <v>0.9</v>
-      </c>
-      <c r="AB25">
-        <f t="shared" si="2"/>
         <v>0.9</v>
       </c>
     </row>

</xml_diff>

<commit_message>
In-progress edits for retirements redesign
</commit_message>
<xml_diff>
--- a/InputData/elec/RAF/Regional Availability Factor.xlsx
+++ b/InputData/elec/RAF/Regional Availability Factor.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MeganMahajan\Documents\eps-us-dev-sandbox\InputData\elec\RAF\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A0AEAB7-2D16-453A-B4D3-25ACC862D5E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB56CAB2-6239-4ED1-B74E-3A7D68FFCF6D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-23820" yWindow="3465" windowWidth="21600" windowHeight="12645" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
+    <workbookView xWindow="2055" yWindow="3375" windowWidth="21600" windowHeight="12645" xr2:uid="{D718C537-5235-45E1-A117-07B097D2BDF0}"/>
   </bookViews>
   <sheets>
     <sheet name="About" sheetId="1" r:id="rId1"/>
@@ -153,7 +153,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="64" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="64">
   <si>
     <t>Source:</t>
   </si>
@@ -342,6 +342,9 @@
   </si>
   <si>
     <t>natural gas combined cycle</t>
+  </si>
+  <si>
+    <t>Update 2026-08-18: natural gas peaker and petroleum RAF set to 0.8 (were 1.0 since 2026-08-17). SYSHECF for these sources calibrates to EIA CF / 0.8 so realized CFs are unchanged at observed EIA levels.</t>
   </si>
 </sst>
 </file>
@@ -897,7 +900,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{667665C7-8A8E-46D9-B686-64BA7741F669}">
-  <dimension ref="A1:B41"/>
+  <dimension ref="A1:B43"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="73.85546875" customWidth="1"/>
@@ -1079,6 +1082,11 @@
     <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>58</v>
+      </c>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2016,82 +2024,82 @@
         <v>10</v>
       </c>
       <c r="B12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="C12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="D12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="J12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="K12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="L12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="M12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="N12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="O12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="P12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Q12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="R12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="S12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="T12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="U12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="V12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="W12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="X12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Y12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Z12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="AA12">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="13" spans="1:27" x14ac:dyDescent="0.25">
@@ -2099,82 +2107,82 @@
         <v>11</v>
       </c>
       <c r="B13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="C13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="D13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="E13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="F13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="G13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="I13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="J13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="K13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="L13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="M13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="N13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="O13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="P13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Q13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="R13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="S13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="T13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="U13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="V13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="W13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="X13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Y13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="Z13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="AA13">
-        <v>1</v>
+        <v>0.8</v>
       </c>
     </row>
     <row r="14" spans="1:27" x14ac:dyDescent="0.25">

</xml_diff>